<commit_message>
Update vendor upload template to include contact information
Add contact name, role, email, phone, and territory columns to the main vendor tab of the Vendor Upload Template.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 9b9a32aa-a5b2-49e8-8fb0-440758a76aee
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 234304c2-50bd-4a44-92af-1c0eca1da560
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Vendor_Upload_Template.xlsx
+++ b/Vendor_Upload_Template.xlsx
@@ -4,7 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Vendors" sheetId="1" r:id="rId1"/>
-    <sheet name="Contacts" sheetId="2" r:id="rId2"/>
+    <sheet name="Additional Contacts" sheetId="2" r:id="rId2"/>
     <sheet name="Logistics &amp; Pricing" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,20 +399,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:Q10"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
     <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="28.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
     <col min="6" max="6" width="38.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
     <col min="8" max="8" width="18.83203125" customWidth="1"/>
     <col min="9" max="9" width="25.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="35.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="25.83203125" customWidth="1"/>
+    <col min="13" max="13" width="22.83203125" customWidth="1"/>
+    <col min="14" max="14" width="32.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
+    <col min="17" max="17" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,12 +455,27 @@
         <v>tags</v>
       </c>
       <c r="L1" t="str">
+        <v>primary_contact_name</v>
+      </c>
+      <c r="M1" t="str">
+        <v>primary_contact_role</v>
+      </c>
+      <c r="N1" t="str">
+        <v>primary_contact_email</v>
+      </c>
+      <c r="O1" t="str">
+        <v>primary_contact_phone</v>
+      </c>
+      <c r="P1" t="str">
+        <v>primary_contact_territory</v>
+      </c>
+      <c r="Q1" t="str">
         <v>notes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>INSTRUCTIONS → short_code is the permanent ID. Use on re-uploads to UPDATE existing records. Leave blank for new records.</v>
+        <v>INSTRUCTIONS → short_code is the permanent ID. Use on re-uploads to UPDATE existing records. Leave blank for new records (system assigns one).</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -488,12 +508,27 @@
         <v/>
       </c>
       <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>INSTRUCTIONS → manufacturer_short_codes: comma-separated list of mfr short_codes this vendor REPS (must match short_code column in Manufacturer template)</v>
+        <v>INSTRUCTIONS → manufacturer_short_codes: comma-separated mfr short_codes this vendor reps — must match short_code column in the Manufacturer template.</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -526,12 +561,27 @@
         <v/>
       </c>
       <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>INSTRUCTIONS → scopes: comma-separated from: accessories, partitions, lockers, corner_guards, wall_protection, signage, fec</v>
+        <v>INSTRUCTIONS → scopes: accessories, partitions, lockers, corner_guards, wall_protection, signage, fec  (comma-separated)</v>
       </c>
       <c r="B4" t="str">
         <v/>
@@ -564,12 +614,27 @@
         <v/>
       </c>
       <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>INSTRUCTIONS → manufacturer_direct: YES if vendor sells direct (no rep). Otherwise NO.</v>
+        <v>INSTRUCTIONS → manufacturer_direct: YES if vendor sells direct from factory, NO if they are a rep or distributor.</v>
       </c>
       <c r="B5" t="str">
         <v/>
@@ -602,12 +667,27 @@
         <v/>
       </c>
       <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>INSTRUCTIONS → category: e.g. Rep Agency, Distributor, Dealer, Manufacturer Direct</v>
+        <v>INSTRUCTIONS → category: Rep Agency | Distributor | Dealer | Manufacturer Direct</v>
       </c>
       <c r="B6" t="str">
         <v/>
@@ -640,6 +720,21 @@
         <v/>
       </c>
       <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
         <v/>
       </c>
     </row>
@@ -678,6 +773,21 @@
         <v/>
       </c>
       <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
         <v/>
       </c>
     </row>
@@ -716,6 +826,21 @@
         <v/>
       </c>
       <c r="L8" t="str">
+        <v>John Ramirez</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Outside Rep</v>
+      </c>
+      <c r="N8" t="str">
+        <v>jramirez@pbspecialties.com</v>
+      </c>
+      <c r="O8" t="str">
+        <v>916-555-0101</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Northern CA</v>
+      </c>
+      <c r="Q8" t="str">
         <v>NorCal + SoCal territory</v>
       </c>
     </row>
@@ -754,6 +879,21 @@
         <v/>
       </c>
       <c r="L9" t="str">
+        <v>Sam Park</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Account Manager</v>
+      </c>
+      <c r="N9" t="str">
+        <v>spark@mcguire.com</v>
+      </c>
+      <c r="O9" t="str">
+        <v>415-555-0301</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Bay Area</v>
+      </c>
+      <c r="Q9" t="str">
         <v/>
       </c>
     </row>
@@ -792,19 +932,34 @@
         <v/>
       </c>
       <c r="L10" t="str">
+        <v>Service Desk</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Customer Service</v>
+      </c>
+      <c r="N10" t="str">
+        <v>service@jlindustries.com</v>
+      </c>
+      <c r="O10" t="str">
+        <v>800-555-0400</v>
+      </c>
+      <c r="P10" t="str">
+        <v>National</v>
+      </c>
+      <c r="Q10" t="str">
         <v>Ships direct from factory</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:G7"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -812,8 +967,7 @@
     <col min="4" max="4" width="32.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="40.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -836,15 +990,12 @@
         <v>territory</v>
       </c>
       <c r="G1" t="str">
-        <v>is_primary</v>
-      </c>
-      <c r="H1" t="str">
         <v>notes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>INSTRUCTIONS → vendor_short_code must match a short_code from the Vendors tab. One row per contact per vendor.</v>
+        <v>INSTRUCTIONS → Use this tab for ADDITIONAL contacts only. The primary contact goes on the Vendors tab.</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -862,15 +1013,12 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>INSTRUCTIONS → is_primary: YES for main contact, NO for additional contacts.</v>
+        <v>INSTRUCTIONS → vendor_short_code must match a short_code from the Vendors tab.</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -888,15 +1036,12 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>INSTRUCTIONS → role: e.g. Inside Sales, Outside Rep, Customer Service, Estimating, Accounting</v>
+        <v>INSTRUCTIONS → role: Inside Sales | Outside Rep | Customer Service | Estimating | Accounting | PM</v>
       </c>
       <c r="B4" t="str">
         <v/>
@@ -914,9 +1059,6 @@
         <v/>
       </c>
       <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
         <v/>
       </c>
     </row>
@@ -940,9 +1082,6 @@
         <v/>
       </c>
       <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
         <v/>
       </c>
     </row>
@@ -951,25 +1090,22 @@
         <v>PBS</v>
       </c>
       <c r="B6" t="str">
-        <v>John Ramirez</v>
+        <v>Maria Lena</v>
       </c>
       <c r="C6" t="str">
-        <v>Outside Rep</v>
+        <v>Inside Sales</v>
       </c>
       <c r="D6" t="str">
-        <v>jramirez@pbspecialties.com</v>
+        <v>mlena@pbspecialties.com</v>
       </c>
       <c r="E6" t="str">
-        <v>916-555-0101</v>
+        <v>916-555-0102</v>
       </c>
       <c r="F6" t="str">
         <v>Northern CA</v>
       </c>
       <c r="G6" t="str">
-        <v>YES</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Main contact for NorCal bids</v>
+        <v>Quote requests + order tracking</v>
       </c>
     </row>
     <row r="7">
@@ -977,108 +1113,27 @@
         <v>PBS</v>
       </c>
       <c r="B7" t="str">
-        <v>Maria Lena</v>
+        <v>Tom Walsh</v>
       </c>
       <c r="C7" t="str">
-        <v>Inside Sales</v>
+        <v>Outside Rep</v>
       </c>
       <c r="D7" t="str">
-        <v>mlena@pbspecialties.com</v>
+        <v>twalsh@pbspecialties.com</v>
       </c>
       <c r="E7" t="str">
-        <v>916-555-0102</v>
+        <v>310-555-0201</v>
       </c>
       <c r="F7" t="str">
-        <v>Northern CA</v>
+        <v>Southern CA</v>
       </c>
       <c r="G7" t="str">
-        <v>NO</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Quote requests + order tracking</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>PBS</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Tom Walsh</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Outside Rep</v>
-      </c>
-      <c r="D8" t="str">
-        <v>twalsh@pbspecialties.com</v>
-      </c>
-      <c r="E8" t="str">
-        <v>310-555-0201</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Southern CA</v>
-      </c>
-      <c r="G8" t="str">
-        <v>NO</v>
-      </c>
-      <c r="H8" t="str">
         <v>SoCal territory</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>MCG</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Sam Park</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Account Manager</v>
-      </c>
-      <c r="D9" t="str">
-        <v>spark@mcguire.com</v>
-      </c>
-      <c r="E9" t="str">
-        <v>415-555-0301</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Bay Area</v>
-      </c>
-      <c r="G9" t="str">
-        <v>YES</v>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>JLI</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Service Desk</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Customer Service</v>
-      </c>
-      <c r="D10" t="str">
-        <v>service@jlindustries.com</v>
-      </c>
-      <c r="E10" t="str">
-        <v>800-555-0400</v>
-      </c>
-      <c r="F10" t="str">
-        <v>National</v>
-      </c>
-      <c r="G10" t="str">
-        <v>YES</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Use for all freight + order questions</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1144,7 +1199,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>INSTRUCTIONS → discount_tier: e.g. Tier 1, Tier 2, Net 30, 40%, 50/10 — however vendor structures it.</v>
+        <v>INSTRUCTIONS → discount_tier: e.g. Tier 1, 50%, 40/10, Net Cost — however vendor structures it.</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -1167,7 +1222,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>INSTRUCTIONS → payment_terms: e.g. Net 30, Net 60, 2% 10 Net 30, Credit Card</v>
+        <v>INSTRUCTIONS → payment_terms: e.g. Net 30, Net 60, 2% 10 Net 30, Credit Card, Pre-pay</v>
       </c>
       <c r="B4" t="str">
         <v/>
@@ -1225,7 +1280,7 @@
         <v>FOB Origin — freight on NBS unless order &gt;$5K</v>
       </c>
       <c r="E6" t="str">
-        <v>Tier 2 / 50%</v>
+        <v>50%</v>
       </c>
       <c r="F6" t="str">
         <v>Net 30</v>

</xml_diff>